<commit_message>
Publish saved example results without input datasets and fix notebook styling
</commit_message>
<xml_diff>
--- a/example/reference_results/8_microbial_load_correction/microbial_load_correction_summary.xlsx
+++ b/example/reference_results/8_microbial_load_correction/microbial_load_correction_summary.xlsx
@@ -246,7 +246,7 @@
     <t xml:space="preserve">2026-09-29 17:44:10 CEST</t>
   </si>
   <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/7_copy_number_correction/copy_number_corrected_asv_count_table.csv</t>
+    <t xml:space="preserve">example/run_results/7_copy_number_correction/copy_number_corrected_asv_count_table.csv</t>
   </si>
   <si>
     <t xml:space="preserve">3b890108568d42995e867a47568550b0</t>
@@ -255,7 +255,7 @@
     <t xml:space="preserve">44ddd7389de9229f9cbce00fb188e4ae</t>
   </si>
   <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/data/cell_count/cell_count.tsv</t>
+    <t xml:space="preserve">example/data/cell_count/cell_count.tsv</t>
   </si>
   <si>
     <t xml:space="preserve">53d33cf33ee93f675d7faffb67a6de04</t>

</xml_diff>